<commit_message>
created sp173178 file and updated it
</commit_message>
<xml_diff>
--- a/July/01.07.2026/book1.xlsx
+++ b/July/01.07.2026/book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/surajsonu07/Desktop/data-analytics/July/01.07.2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C37746F-068E-7D40-9B76-41B10FDE47A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B934D14-D5D5-7543-A111-2E76C8D23A6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32340" yWindow="1020" windowWidth="30880" windowHeight="16920" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,6 +20,16 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$A$2:$A$7</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$B$1</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$B$2:$B$7</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$C$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$C$2:$C$7</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$A$2:$A$7</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet2!$B$1</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet2!$B$2:$B$7</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Sheet2!$C$1</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Sheet2!$C$2:$C$7</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">'customers'!$A$1:$K$93</definedName>
     <definedName name="ExternalData_2" localSheetId="0" hidden="1">products!$A$1:$K$78</definedName>
   </definedNames>
@@ -52,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="966">
   <si>
     <t>Item_id</t>
   </si>
@@ -2917,6 +2927,39 @@
   </si>
   <si>
     <t>Sales Report</t>
+  </si>
+  <si>
+    <t>sp173</t>
+  </si>
+  <si>
+    <t>Area Chart</t>
+  </si>
+  <si>
+    <t>sp174</t>
+  </si>
+  <si>
+    <t>Surface Chart</t>
+  </si>
+  <si>
+    <t>sp175</t>
+  </si>
+  <si>
+    <t>Radar Chart</t>
+  </si>
+  <si>
+    <t>sp176</t>
+  </si>
+  <si>
+    <t>Bubble Chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>sp178</t>
+  </si>
+  <si>
+    <t>Stock Chart</t>
   </si>
 </sst>
 </file>
@@ -4319,7 +4362,2237 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>Sheet2!$B$20</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>Area Chart</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:areaChart>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2021-2022</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3453</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45345</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4345</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5435</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54324</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5643</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A3BB-1E4A-9CE2-F93C6BF7260E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2022-2023</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>6543</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34553</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45343</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34234</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2345</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>543</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A3BB-1E4A-9CE2-F93C6BF7260E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1040523583"/>
+        <c:axId val="1037149823"/>
+      </c:areaChart>
+      <c:catAx>
+        <c:axId val="1040523583"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037149823"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1037149823"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1040523583"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>Sheet2!$B$21</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>Surface Chart</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="15"/>
+      <c:rotY val="20"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:surface3DChart>
+        <c:wireframe val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2021-2022</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln/>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3453</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45345</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4345</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5435</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54324</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5643</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-066C-8144-BF95-73AA3A8FE513}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2022-2023</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln/>
+            <a:effectLst/>
+            <a:sp3d/>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>6543</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34553</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45343</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34234</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2345</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>543</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-066C-8144-BF95-73AA3A8FE513}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:bandFmts>
+          <c:bandFmt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="3"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="4"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="9"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="11"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="12"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="13"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+          <c:bandFmt>
+            <c:idx val="14"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln/>
+              <a:effectLst/>
+              <a:sp3d/>
+            </c:spPr>
+          </c:bandFmt>
+        </c:bandFmts>
+        <c:axId val="1037853887"/>
+        <c:axId val="1037859711"/>
+        <c:axId val="1039083007"/>
+      </c:surface3DChart>
+      <c:catAx>
+        <c:axId val="1037853887"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037859711"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1037859711"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037853887"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:serAx>
+        <c:axId val="1039083007"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037859711"/>
+        <c:crosses val="autoZero"/>
+      </c:serAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>Sheet2!$B$22</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>Radar Chart</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2021-2022</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3453</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45345</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4345</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5435</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54324</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5643</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5AD8-B043-B96D-3E1E9DD6E101}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2022-2023</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>6543</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34553</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45343</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34234</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2345</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>543</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5AD8-B043-B96D-3E1E9DD6E101}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1037421631"/>
+        <c:axId val="1037424767"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="1037421631"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037424767"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1037424767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037421631"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:strRef>
+          <c:f>Sheet2!$B$23</c:f>
+          <c:strCache>
+            <c:ptCount val="1"/>
+            <c:pt idx="0">
+              <c:v>Bubble Chart</c:v>
+            </c:pt>
+          </c:strCache>
+        </c:strRef>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:bubbleChart>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2021-2022</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx2"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="tx2">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Watch</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Bike</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Phone</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Laptop Changer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3453</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45345</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4345</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5435</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>54324</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5643</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:bubbleSize>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>6543</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34553</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45343</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34234</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2345</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>543</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:bubbleSize>
+          <c:bubble3D val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8575-C549-8EBF-5FE88DBCCFC9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:bubbleScale val="100"/>
+        <c:showNegBubbles val="0"/>
+        <c:axId val="1037145343"/>
+        <c:axId val="1038320063"/>
+      </c:bubbleChart>
+      <c:valAx>
+        <c:axId val="1037145343"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx2">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1038320063"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1038320063"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx2">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx2"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1037145343"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx2">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.2</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.4</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Stock Chart</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Stock Chart</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="waterfall" uniqueId="{00000000-1A1C-BC49-8F47-D607CA5AFF32}" formatIdx="0">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:v>2021-2022</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataLabels pos="outEnd">
+            <cx:visibility seriesName="0" categoryName="0" value="1"/>
+          </cx:dataLabels>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:subtotals/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="waterfall" hidden="1" uniqueId="{00000001-1A1C-BC49-8F47-D607CA5AFF32}" formatIdx="1">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.3</cx:f>
+              <cx:v>2022-2023</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataLabels pos="outEnd">
+            <cx:visibility seriesName="0" categoryName="0" value="1"/>
+          </cx:dataLabels>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:subtotals/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="t" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4862,20 +7135,2033 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="276">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="317">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="242">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk2">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="395">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>266700</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>673100</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>165100</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4898,6 +9184,228 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>806450</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3C2EAFC-1FFA-D980-928B-BD9582B0CB78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>177800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>387350</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB487582-BBFF-4F36-5A44-3A11F993DDB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>615950</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>234950</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5E43B55-7FBD-F3DD-1502-D7E4E04FB831}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>596900</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>336550</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0801157-483B-7BEC-3F0A-9F2D059A91DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>336550</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>781050</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="9" name="Chart 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A74B4D6-8591-B621-5EAB-F732E7A7A686}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2990850" y="3943350"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-GB" sz="1100"/>
+                <a:t>This chart isn’t available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -11375,7 +15883,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11F1A1C1-E3B8-364E-9A58-899ED026CCCC}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -11489,20 +15997,68 @@
         <v>950</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>951</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>952</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>953</v>
       </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>955</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>957</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>959</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>961</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>964</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B26" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>